<commit_message>
feat: complete planner chart tooling and pending game integrations
</commit_message>
<xml_diff>
--- a/tools/planner-studio/app/seeds/PermanentUpgrade.xlsx
+++ b/tools/planner-studio/app/seeds/PermanentUpgrade.xlsx
@@ -143,50 +143,55 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t xml:space="preserve">IconAddress</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Shape</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t xml:space="preserve">MaxLevel</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t xml:space="preserve">ValuePerLevel</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t xml:space="preserve">Row</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t xml:space="preserve">Column</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t xml:space="preserve">Parents</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t xml:space="preserve">RequireAnyParent</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t xml:space="preserve">RequiredTotalLevel</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t xml:space="preserve">ExclusiveGroup</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t xml:space="preserve">RecommendOrder</t>
         </is>
@@ -215,38 +220,43 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F2">
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G2">
         <v>3</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>0.002</v>
       </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
       <c r="I2">
         <v>0</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K2">
-        <v>0</v>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N2">
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O2">
         <v>0</v>
       </c>
     </row>
@@ -273,38 +283,43 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F3">
+          <t xml:space="preserve">Research/Icons/e0d9939b4e24549aebfe1441f4104b8b[PictoIcon_Critical]</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G3">
         <v>3</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>0.001</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>1</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>-1</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">1-1</t>
         </is>
       </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
       <c r="L3">
         <v>0</v>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N3">
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O3">
         <v>0</v>
       </c>
     </row>
@@ -331,38 +346,43 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F4">
+          <t xml:space="preserve">Research/Icons/9851fb8e6f12a40d09379e3d9a144449[PictoIcon_Thunder]</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G4">
         <v>3</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>0.003</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t xml:space="preserve">1-1</t>
         </is>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
       <c r="L4">
         <v>0</v>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N4">
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O4">
         <v>0</v>
       </c>
     </row>
@@ -389,38 +409,43 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F5">
+          <t xml:space="preserve">Research/Icons/9df0f4d8c02014347ad2d7de427e0ced[Star Filled]</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G5">
         <v>3</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>0.003</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>2</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>-1</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t xml:space="preserve">2-1</t>
         </is>
       </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
       <c r="L5">
         <v>0</v>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N5">
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O5">
         <v>0</v>
       </c>
     </row>
@@ -447,38 +472,43 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F6">
+          <t xml:space="preserve">Research/Icons/447cb81759d8742888a02fa6be150fd0[PictoIcon_Support]</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G6">
         <v>3</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>0.002</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>2</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t xml:space="preserve">2-2</t>
         </is>
       </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
       <c r="L6">
         <v>0</v>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N6">
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O6">
         <v>0</v>
       </c>
     </row>
@@ -505,38 +535,43 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Circle</t>
         </is>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>5</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>0.002</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>3</v>
       </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t xml:space="preserve">3-1;3-2</t>
         </is>
       </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
       <c r="L7">
         <v>0</v>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N7">
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O7">
         <v>0</v>
       </c>
     </row>
@@ -563,38 +598,43 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/038ccab8cd184d04cb1bfa1d79704320[Medal]</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Special</t>
         </is>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>1</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>0.015</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>3</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>2</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t xml:space="preserve">4-1</t>
         </is>
       </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
       <c r="L8">
         <v>0</v>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N8">
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O8">
         <v>0</v>
       </c>
     </row>
@@ -621,38 +661,43 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F9">
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G9">
         <v>5</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>0.002</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>4</v>
       </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t xml:space="preserve">4-1</t>
         </is>
       </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
       <c r="L9">
         <v>0</v>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N9">
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O9">
         <v>0</v>
       </c>
     </row>
@@ -679,38 +724,43 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F10">
+          <t xml:space="preserve">Research/Icons/1e41e49e206bc2947b8943351eed53d3[Clock]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G10">
         <v>5</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>0.002</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>5</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>-1</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t xml:space="preserve">5-1</t>
         </is>
       </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
       <c r="L10">
         <v>0</v>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N10">
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O10">
         <v>0</v>
       </c>
     </row>
@@ -737,38 +787,43 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F11">
+          <t xml:space="preserve">Research/Icons/a5edbb1acb3234a5db0f0daa141eb77b[PictoIcon_Fire]</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G11">
         <v>5</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>0.004</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>5</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t xml:space="preserve">5-1</t>
         </is>
       </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
       <c r="L11">
         <v>0</v>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N11">
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O11">
         <v>0</v>
       </c>
     </row>
@@ -795,38 +850,43 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F12">
+          <t xml:space="preserve">Research/Icons/f5d3c19ee35f34a7dae4a36e5ec57472[PictoIcon_Boss]</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G12">
         <v>5</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>0.003</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>6</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>-1</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t xml:space="preserve">6-1</t>
         </is>
       </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
       <c r="L12">
         <v>0</v>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N12">
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O12">
         <v>0</v>
       </c>
     </row>
@@ -853,38 +913,43 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F13">
+          <t xml:space="preserve">Research/Icons/e7f5d551fd1925040bd01a8ec66c0ae0[Store Bag]</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G13">
         <v>5</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>3</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>6</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>1</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t xml:space="preserve">6-2</t>
         </is>
       </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
       <c r="L13">
         <v>0</v>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N13">
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O13">
         <v>0</v>
       </c>
     </row>
@@ -911,38 +976,43 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t xml:space="preserve">Circle</t>
         </is>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>7</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>0.002</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>7</v>
       </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr">
         <is>
           <t xml:space="preserve">7-1;7-2</t>
         </is>
       </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
       <c r="L14">
         <v>0</v>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N14">
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O14">
         <v>0</v>
       </c>
     </row>
@@ -969,38 +1039,43 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/038ccab8cd184d04cb1bfa1d79704320[Medal]</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t xml:space="preserve">Special</t>
         </is>
       </c>
-      <c r="F15">
+      <c r="G15">
         <v>1</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>5</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>7</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>2</v>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t xml:space="preserve">8-1</t>
         </is>
       </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
       <c r="L15">
         <v>0</v>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N15">
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O15">
         <v>0</v>
       </c>
     </row>
@@ -1027,38 +1102,43 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F16">
+          <t xml:space="preserve">Research/Icons/12ce67a96878541b29388f9452483249[PictoIcon_Temple]</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G16">
         <v>7</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>0.002</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>8</v>
       </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16" t="inlineStr">
         <is>
           <t xml:space="preserve">8-1</t>
         </is>
       </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
       <c r="L16">
         <v>0</v>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N16">
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O16">
         <v>0</v>
       </c>
     </row>
@@ -1085,38 +1165,43 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F17">
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G17">
         <v>7</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>0.002</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>9</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>-1</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t xml:space="preserve">9-1</t>
         </is>
       </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
       <c r="L17">
         <v>0</v>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N17">
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O17">
         <v>0</v>
       </c>
     </row>
@@ -1143,38 +1228,43 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F18">
+          <t xml:space="preserve">Research/Icons/e0d9939b4e24549aebfe1441f4104b8b[PictoIcon_Critical]</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G18">
         <v>7</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>0.001</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>9</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>1</v>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t xml:space="preserve">9-1</t>
         </is>
       </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
       <c r="L18">
         <v>0</v>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N18">
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O18">
         <v>0</v>
       </c>
     </row>
@@ -1201,38 +1291,43 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F19">
+          <t xml:space="preserve">Research/Icons/9851fb8e6f12a40d09379e3d9a144449[PictoIcon_Thunder]</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G19">
         <v>7</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <v>0.003</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>10</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>-1</v>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t xml:space="preserve">10-1</t>
         </is>
       </c>
-      <c r="K19">
-        <v>0</v>
-      </c>
       <c r="L19">
         <v>0</v>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N19">
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O19">
         <v>0</v>
       </c>
     </row>
@@ -1259,38 +1354,43 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F20">
+          <t xml:space="preserve">Research/Icons/9df0f4d8c02014347ad2d7de427e0ced[Star Filled]</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G20">
         <v>7</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <v>0.003</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>10</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>1</v>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t xml:space="preserve">10-2</t>
         </is>
       </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
       <c r="L20">
         <v>0</v>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N20">
+      <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O20">
         <v>0</v>
       </c>
     </row>
@@ -1317,38 +1417,43 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t xml:space="preserve">Circle</t>
         </is>
       </c>
-      <c r="F21">
+      <c r="G21">
         <v>9</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>0.002</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>11</v>
       </c>
-      <c r="I21">
-        <v>0</v>
-      </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr">
         <is>
           <t xml:space="preserve">11-1;11-2</t>
         </is>
       </c>
-      <c r="K21">
-        <v>0</v>
-      </c>
       <c r="L21">
         <v>0</v>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N21">
+      <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O21">
         <v>0</v>
       </c>
     </row>
@@ -1375,38 +1480,43 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/038ccab8cd184d04cb1bfa1d79704320[Medal]</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t xml:space="preserve">Special</t>
         </is>
       </c>
-      <c r="F22">
+      <c r="G22">
         <v>1</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>0.01</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>11</v>
       </c>
-      <c r="I22">
+      <c r="J22">
         <v>2</v>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t xml:space="preserve">12-1</t>
         </is>
       </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
       <c r="L22">
         <v>0</v>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N22">
+      <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O22">
         <v>0</v>
       </c>
     </row>
@@ -1433,38 +1543,43 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F23">
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G23">
         <v>3</v>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>0.02</v>
       </c>
-      <c r="H23">
-        <v>0</v>
-      </c>
       <c r="I23">
         <v>0</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K23">
-        <v>0</v>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="L23">
         <v>0</v>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N23">
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O23">
         <v>1</v>
       </c>
     </row>
@@ -1491,38 +1606,43 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F24">
+          <t xml:space="preserve">Research/Icons/e0d9939b4e24549aebfe1441f4104b8b[PictoIcon_Critical]</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G24">
         <v>3</v>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>0.02</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>1</v>
       </c>
-      <c r="I24">
+      <c r="J24">
         <v>-1</v>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="K24">
-        <v>0</v>
-      </c>
       <c r="L24">
         <v>0</v>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24" t="inlineStr">
         <is>
           <t xml:space="preserve">choice1</t>
         </is>
       </c>
-      <c r="N24">
+      <c r="O24">
         <v>11</v>
       </c>
     </row>
@@ -1549,38 +1669,43 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F25">
+          <t xml:space="preserve">Research/Icons/9851fb8e6f12a40d09379e3d9a144449[PictoIcon_Thunder]</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G25">
         <v>3</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>0.02</v>
-      </c>
-      <c r="H25">
-        <v>1</v>
       </c>
       <c r="I25">
         <v>1</v>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J25">
+        <v>1</v>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
       <c r="L25">
         <v>0</v>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25" t="inlineStr">
         <is>
           <t xml:space="preserve">choice1</t>
         </is>
       </c>
-      <c r="N25">
+      <c r="O25">
         <v>0</v>
       </c>
     </row>
@@ -1607,38 +1732,43 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t xml:space="preserve">Circle</t>
         </is>
       </c>
-      <c r="F26">
+      <c r="G26">
         <v>5</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>0.02</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>2</v>
       </c>
-      <c r="I26">
-        <v>0</v>
-      </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26" t="inlineStr">
         <is>
           <t xml:space="preserve">2-A;2-B</t>
         </is>
       </c>
-      <c r="K26">
+      <c r="L26">
         <v>1</v>
       </c>
-      <c r="L26">
-        <v>0</v>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N26">
+      <c r="M26">
+        <v>0</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O26">
         <v>20</v>
       </c>
     </row>
@@ -1665,38 +1795,43 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F27">
+          <t xml:space="preserve">Research/Icons/447cb81759d8742888a02fa6be150fd0[PictoIcon_Support]</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G27">
         <v>3</v>
       </c>
-      <c r="G27">
+      <c r="H27">
         <v>0.02</v>
       </c>
-      <c r="H27">
+      <c r="I27">
         <v>3</v>
       </c>
-      <c r="I27">
+      <c r="J27">
         <v>-1</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t xml:space="preserve">2-C</t>
         </is>
       </c>
-      <c r="K27">
-        <v>0</v>
-      </c>
       <c r="L27">
         <v>0</v>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M27">
+        <v>0</v>
+      </c>
+      <c r="N27" t="inlineStr">
         <is>
           <t xml:space="preserve">choice2</t>
         </is>
       </c>
-      <c r="N27">
+      <c r="O27">
         <v>31</v>
       </c>
     </row>
@@ -1723,38 +1858,43 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F28">
+          <t xml:space="preserve">Research/Icons/f5d3c19ee35f34a7dae4a36e5ec57472[PictoIcon_Boss]</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G28">
         <v>3</v>
       </c>
-      <c r="G28">
+      <c r="H28">
         <v>0.02</v>
       </c>
-      <c r="H28">
+      <c r="I28">
         <v>3</v>
       </c>
-      <c r="I28">
+      <c r="J28">
         <v>1</v>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t xml:space="preserve">2-C</t>
         </is>
       </c>
-      <c r="K28">
-        <v>0</v>
-      </c>
       <c r="L28">
         <v>0</v>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28" t="inlineStr">
         <is>
           <t xml:space="preserve">choice2</t>
         </is>
       </c>
-      <c r="N28">
+      <c r="O28">
         <v>0</v>
       </c>
     </row>
@@ -1781,38 +1921,43 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/1e41e49e206bc2947b8943351eed53d3[Clock]</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t xml:space="preserve">Circle</t>
         </is>
       </c>
-      <c r="F29">
+      <c r="G29">
         <v>5</v>
       </c>
-      <c r="G29">
+      <c r="H29">
         <v>0.02</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>4</v>
       </c>
-      <c r="I29">
-        <v>0</v>
-      </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29" t="inlineStr">
         <is>
           <t xml:space="preserve">3-A;3-B</t>
         </is>
       </c>
-      <c r="K29">
+      <c r="L29">
         <v>1</v>
       </c>
-      <c r="L29">
-        <v>0</v>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N29">
+      <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O29">
         <v>40</v>
       </c>
     </row>
@@ -1839,38 +1984,43 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F30">
+          <t xml:space="preserve">Research/Icons/a5edbb1acb3234a5db0f0daa141eb77b[PictoIcon_Fire]</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G30">
         <v>3</v>
       </c>
-      <c r="G30">
+      <c r="H30">
         <v>0.02</v>
       </c>
-      <c r="H30">
+      <c r="I30">
         <v>5</v>
       </c>
-      <c r="I30">
+      <c r="J30">
         <v>-1</v>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t xml:space="preserve">3-C</t>
         </is>
       </c>
-      <c r="K30">
-        <v>0</v>
-      </c>
       <c r="L30">
         <v>0</v>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="M30">
+        <v>0</v>
+      </c>
+      <c r="N30" t="inlineStr">
         <is>
           <t xml:space="preserve">choice3</t>
         </is>
       </c>
-      <c r="N30">
+      <c r="O30">
         <v>51</v>
       </c>
     </row>
@@ -1897,38 +2047,43 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F31">
+          <t xml:space="preserve">Research/Icons/9df0f4d8c02014347ad2d7de427e0ced[Star Filled]</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G31">
         <v>3</v>
       </c>
-      <c r="G31">
+      <c r="H31">
         <v>0.02</v>
       </c>
-      <c r="H31">
+      <c r="I31">
         <v>5</v>
       </c>
-      <c r="I31">
+      <c r="J31">
         <v>1</v>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t xml:space="preserve">3-C</t>
         </is>
       </c>
-      <c r="K31">
-        <v>0</v>
-      </c>
       <c r="L31">
         <v>0</v>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M31">
+        <v>0</v>
+      </c>
+      <c r="N31" t="inlineStr">
         <is>
           <t xml:space="preserve">choice3</t>
         </is>
       </c>
-      <c r="N31">
+      <c r="O31">
         <v>0</v>
       </c>
     </row>
@@ -1955,38 +2110,43 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t xml:space="preserve">Circle</t>
         </is>
       </c>
-      <c r="F32">
+      <c r="G32">
         <v>5</v>
       </c>
-      <c r="G32">
+      <c r="H32">
         <v>0.02</v>
       </c>
-      <c r="H32">
+      <c r="I32">
         <v>6</v>
       </c>
-      <c r="I32">
-        <v>0</v>
-      </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32" t="inlineStr">
         <is>
           <t xml:space="preserve">4-A;4-B</t>
         </is>
       </c>
-      <c r="K32">
+      <c r="L32">
         <v>1</v>
       </c>
-      <c r="L32">
-        <v>0</v>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N32">
+      <c r="M32">
+        <v>0</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O32">
         <v>60</v>
       </c>
     </row>
@@ -2013,38 +2173,43 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F33">
+          <t xml:space="preserve">Research/Icons/12ce67a96878541b29388f9452483249[PictoIcon_Temple]</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G33">
         <v>3</v>
       </c>
-      <c r="G33">
+      <c r="H33">
         <v>0.02</v>
       </c>
-      <c r="H33">
+      <c r="I33">
         <v>7</v>
       </c>
-      <c r="I33">
+      <c r="J33">
         <v>-1</v>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t xml:space="preserve">4-C</t>
         </is>
       </c>
-      <c r="K33">
-        <v>0</v>
-      </c>
       <c r="L33">
         <v>0</v>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M33">
+        <v>0</v>
+      </c>
+      <c r="N33" t="inlineStr">
         <is>
           <t xml:space="preserve">choice4</t>
         </is>
       </c>
-      <c r="N33">
+      <c r="O33">
         <v>71</v>
       </c>
     </row>
@@ -2071,38 +2236,43 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F34">
+          <t xml:space="preserve">Research/Icons/e7f5d551fd1925040bd01a8ec66c0ae0[Store Bag]</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G34">
         <v>3</v>
       </c>
-      <c r="G34">
+      <c r="H34">
         <v>30</v>
       </c>
-      <c r="H34">
+      <c r="I34">
         <v>7</v>
       </c>
-      <c r="I34">
+      <c r="J34">
         <v>1</v>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t xml:space="preserve">4-C</t>
         </is>
       </c>
-      <c r="K34">
-        <v>0</v>
-      </c>
       <c r="L34">
         <v>0</v>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M34">
+        <v>0</v>
+      </c>
+      <c r="N34" t="inlineStr">
         <is>
           <t xml:space="preserve">choice4</t>
         </is>
       </c>
-      <c r="N34">
+      <c r="O34">
         <v>0</v>
       </c>
     </row>
@@ -2129,38 +2299,43 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/65a1928224b8541439b433a52ea9c3d9[Cup]</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t xml:space="preserve">Special</t>
         </is>
       </c>
-      <c r="F35">
+      <c r="G35">
         <v>3</v>
       </c>
-      <c r="G35">
+      <c r="H35">
         <v>0.1</v>
       </c>
-      <c r="H35">
+      <c r="I35">
         <v>8</v>
       </c>
-      <c r="I35">
-        <v>0</v>
-      </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35">
+        <v>0</v>
+      </c>
+      <c r="K35" t="inlineStr">
         <is>
           <t xml:space="preserve">5-A;5-B</t>
         </is>
       </c>
-      <c r="K35">
+      <c r="L35">
         <v>1</v>
       </c>
-      <c r="L35">
-        <v>0</v>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N35">
+      <c r="M35">
+        <v>0</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O35">
         <v>80</v>
       </c>
     </row>
@@ -2187,38 +2362,43 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F36">
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G36">
         <v>3</v>
       </c>
-      <c r="G36">
+      <c r="H36">
         <v>0.02</v>
       </c>
-      <c r="H36">
-        <v>0</v>
-      </c>
       <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
         <v>-1</v>
       </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K36">
-        <v>0</v>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="L36">
         <v>0</v>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N36">
+      <c r="M36">
+        <v>0</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O36">
         <v>1</v>
       </c>
     </row>
@@ -2245,38 +2425,43 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F37">
+          <t xml:space="preserve">Research/Icons/e0d9939b4e24549aebfe1441f4104b8b[PictoIcon_Critical]</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G37">
         <v>3</v>
       </c>
-      <c r="G37">
+      <c r="H37">
         <v>0.01</v>
       </c>
-      <c r="H37">
-        <v>0</v>
-      </c>
       <c r="I37">
         <v>0</v>
       </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K37">
-        <v>0</v>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="L37">
         <v>0</v>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N37">
+      <c r="M37">
+        <v>0</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O37">
         <v>2</v>
       </c>
     </row>
@@ -2303,38 +2488,43 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F38">
+          <t xml:space="preserve">Research/Icons/447cb81759d8742888a02fa6be150fd0[PictoIcon_Support]</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G38">
         <v>3</v>
       </c>
-      <c r="G38">
+      <c r="H38">
         <v>0.03</v>
       </c>
-      <c r="H38">
-        <v>0</v>
-      </c>
       <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
         <v>1</v>
       </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K38">
-        <v>0</v>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="L38">
         <v>0</v>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N38">
+      <c r="M38">
+        <v>0</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O38">
         <v>3</v>
       </c>
     </row>
@@ -2361,38 +2551,43 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F39">
+          <t xml:space="preserve">Research/Icons/9851fb8e6f12a40d09379e3d9a144449[PictoIcon_Thunder]</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G39">
         <v>3</v>
       </c>
-      <c r="G39">
+      <c r="H39">
         <v>0.02</v>
       </c>
-      <c r="H39">
+      <c r="I39">
         <v>1</v>
       </c>
-      <c r="I39">
+      <c r="J39">
         <v>-1</v>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t xml:space="preserve">1-L1</t>
         </is>
       </c>
-      <c r="K39">
-        <v>0</v>
-      </c>
       <c r="L39">
         <v>0</v>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N39">
+      <c r="M39">
+        <v>0</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O39">
         <v>4</v>
       </c>
     </row>
@@ -2419,38 +2614,43 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F40">
+          <t xml:space="preserve">Research/Icons/9df0f4d8c02014347ad2d7de427e0ced[Star Filled]</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G40">
         <v>3</v>
       </c>
-      <c r="G40">
+      <c r="H40">
         <v>0.01</v>
       </c>
-      <c r="H40">
+      <c r="I40">
         <v>1</v>
       </c>
-      <c r="I40">
-        <v>0</v>
-      </c>
-      <c r="J40" t="inlineStr">
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40" t="inlineStr">
         <is>
           <t xml:space="preserve">1-M1</t>
         </is>
       </c>
-      <c r="K40">
-        <v>0</v>
-      </c>
       <c r="L40">
         <v>0</v>
       </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N40">
+      <c r="M40">
+        <v>0</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O40">
         <v>5</v>
       </c>
     </row>
@@ -2477,38 +2677,43 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F41">
+          <t xml:space="preserve">Research/Icons/e7f5d551fd1925040bd01a8ec66c0ae0[Store Bag]</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G41">
         <v>3</v>
       </c>
-      <c r="G41">
+      <c r="H41">
         <v>30</v>
-      </c>
-      <c r="H41">
-        <v>1</v>
       </c>
       <c r="I41">
         <v>1</v>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J41">
+        <v>1</v>
+      </c>
+      <c r="K41" t="inlineStr">
         <is>
           <t xml:space="preserve">1-R1</t>
         </is>
       </c>
-      <c r="K41">
-        <v>0</v>
-      </c>
       <c r="L41">
         <v>0</v>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N41">
+      <c r="M41">
+        <v>0</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O41">
         <v>6</v>
       </c>
     </row>
@@ -2535,38 +2740,43 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F42">
+          <t xml:space="preserve">Research/Icons/f5d3c19ee35f34a7dae4a36e5ec57472[PictoIcon_Boss]</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G42">
         <v>3</v>
       </c>
-      <c r="G42">
+      <c r="H42">
         <v>0.02</v>
       </c>
-      <c r="H42">
+      <c r="I42">
         <v>2</v>
       </c>
-      <c r="I42">
+      <c r="J42">
         <v>-1</v>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t xml:space="preserve">1-L2</t>
         </is>
       </c>
-      <c r="K42">
-        <v>0</v>
-      </c>
       <c r="L42">
         <v>0</v>
       </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N42">
+      <c r="M42">
+        <v>0</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O42">
         <v>7</v>
       </c>
     </row>
@@ -2593,38 +2803,43 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F43">
+          <t xml:space="preserve">Research/Icons/a5edbb1acb3234a5db0f0daa141eb77b[PictoIcon_Fire]</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G43">
         <v>3</v>
       </c>
-      <c r="G43">
+      <c r="H43">
         <v>0.01</v>
       </c>
-      <c r="H43">
+      <c r="I43">
         <v>2</v>
       </c>
-      <c r="I43">
-        <v>0</v>
-      </c>
-      <c r="J43" t="inlineStr">
+      <c r="J43">
+        <v>0</v>
+      </c>
+      <c r="K43" t="inlineStr">
         <is>
           <t xml:space="preserve">1-M2</t>
         </is>
       </c>
-      <c r="K43">
-        <v>0</v>
-      </c>
       <c r="L43">
         <v>0</v>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N43">
+      <c r="M43">
+        <v>0</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O43">
         <v>8</v>
       </c>
     </row>
@@ -2651,38 +2866,43 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F44">
+          <t xml:space="preserve">Research/Icons/1e41e49e206bc2947b8943351eed53d3[Clock]</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G44">
         <v>3</v>
       </c>
-      <c r="G44">
+      <c r="H44">
         <v>0.03</v>
       </c>
-      <c r="H44">
+      <c r="I44">
         <v>2</v>
       </c>
-      <c r="I44">
+      <c r="J44">
         <v>1</v>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t xml:space="preserve">1-R2</t>
         </is>
       </c>
-      <c r="K44">
-        <v>0</v>
-      </c>
       <c r="L44">
         <v>0</v>
       </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N44">
+      <c r="M44">
+        <v>0</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O44">
         <v>9</v>
       </c>
     </row>
@@ -2709,38 +2929,43 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/038ccab8cd184d04cb1bfa1d79704320[Medal]</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
           <t xml:space="preserve">Circle</t>
         </is>
       </c>
-      <c r="F45">
+      <c r="G45">
         <v>1</v>
       </c>
-      <c r="G45">
+      <c r="H45">
         <v>0.05</v>
       </c>
-      <c r="H45">
+      <c r="I45">
         <v>3</v>
       </c>
-      <c r="I45">
-        <v>0</v>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K45">
-        <v>0</v>
+      <c r="J45">
+        <v>0</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="L45">
+        <v>0</v>
+      </c>
+      <c r="M45">
         <v>12</v>
       </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N45">
+      <c r="N45" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O45">
         <v>11</v>
       </c>
     </row>
@@ -2767,38 +2992,43 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F46">
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G46">
         <v>5</v>
       </c>
-      <c r="G46">
+      <c r="H46">
         <v>0.02</v>
       </c>
-      <c r="H46">
+      <c r="I46">
         <v>4</v>
       </c>
-      <c r="I46">
+      <c r="J46">
         <v>-1</v>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t xml:space="preserve">G1</t>
         </is>
       </c>
-      <c r="K46">
-        <v>0</v>
-      </c>
       <c r="L46">
         <v>0</v>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N46">
+      <c r="M46">
+        <v>0</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O46">
         <v>13</v>
       </c>
     </row>
@@ -2825,38 +3055,43 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F47">
+          <t xml:space="preserve">Research/Icons/e0d9939b4e24549aebfe1441f4104b8b[PictoIcon_Critical]</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G47">
         <v>5</v>
       </c>
-      <c r="G47">
+      <c r="H47">
         <v>0.01</v>
       </c>
-      <c r="H47">
+      <c r="I47">
         <v>4</v>
       </c>
-      <c r="I47">
-        <v>0</v>
-      </c>
-      <c r="J47" t="inlineStr">
+      <c r="J47">
+        <v>0</v>
+      </c>
+      <c r="K47" t="inlineStr">
         <is>
           <t xml:space="preserve">G1</t>
         </is>
       </c>
-      <c r="K47">
-        <v>0</v>
-      </c>
       <c r="L47">
         <v>0</v>
       </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N47">
+      <c r="M47">
+        <v>0</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O47">
         <v>14</v>
       </c>
     </row>
@@ -2883,38 +3118,43 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F48">
+          <t xml:space="preserve">Research/Icons/447cb81759d8742888a02fa6be150fd0[PictoIcon_Support]</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G48">
         <v>5</v>
       </c>
-      <c r="G48">
+      <c r="H48">
         <v>0.03</v>
       </c>
-      <c r="H48">
+      <c r="I48">
         <v>4</v>
       </c>
-      <c r="I48">
+      <c r="J48">
         <v>1</v>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t xml:space="preserve">G1</t>
         </is>
       </c>
-      <c r="K48">
-        <v>0</v>
-      </c>
       <c r="L48">
         <v>0</v>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N48">
+      <c r="M48">
+        <v>0</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O48">
         <v>15</v>
       </c>
     </row>
@@ -2941,38 +3181,43 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F49">
+          <t xml:space="preserve">Research/Icons/9851fb8e6f12a40d09379e3d9a144449[PictoIcon_Thunder]</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G49">
         <v>5</v>
       </c>
-      <c r="G49">
+      <c r="H49">
         <v>0.02</v>
       </c>
-      <c r="H49">
+      <c r="I49">
         <v>5</v>
       </c>
-      <c r="I49">
+      <c r="J49">
         <v>-1</v>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t xml:space="preserve">2-L1</t>
         </is>
       </c>
-      <c r="K49">
-        <v>0</v>
-      </c>
       <c r="L49">
         <v>0</v>
       </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N49">
+      <c r="M49">
+        <v>0</v>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O49">
         <v>16</v>
       </c>
     </row>
@@ -2999,38 +3244,43 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F50">
+          <t xml:space="preserve">Research/Icons/9df0f4d8c02014347ad2d7de427e0ced[Star Filled]</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G50">
         <v>5</v>
       </c>
-      <c r="G50">
+      <c r="H50">
         <v>0.01</v>
       </c>
-      <c r="H50">
+      <c r="I50">
         <v>5</v>
       </c>
-      <c r="I50">
-        <v>0</v>
-      </c>
-      <c r="J50" t="inlineStr">
+      <c r="J50">
+        <v>0</v>
+      </c>
+      <c r="K50" t="inlineStr">
         <is>
           <t xml:space="preserve">2-M1</t>
         </is>
       </c>
-      <c r="K50">
-        <v>0</v>
-      </c>
       <c r="L50">
         <v>0</v>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N50">
+      <c r="M50">
+        <v>0</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O50">
         <v>17</v>
       </c>
     </row>
@@ -3057,38 +3307,43 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F51">
+          <t xml:space="preserve">Research/Icons/e7f5d551fd1925040bd01a8ec66c0ae0[Store Bag]</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G51">
         <v>5</v>
       </c>
-      <c r="G51">
+      <c r="H51">
         <v>30</v>
       </c>
-      <c r="H51">
+      <c r="I51">
         <v>5</v>
       </c>
-      <c r="I51">
+      <c r="J51">
         <v>1</v>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t xml:space="preserve">2-R1</t>
         </is>
       </c>
-      <c r="K51">
-        <v>0</v>
-      </c>
       <c r="L51">
         <v>0</v>
       </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N51">
+      <c r="M51">
+        <v>0</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O51">
         <v>18</v>
       </c>
     </row>
@@ -3115,38 +3370,43 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F52">
+          <t xml:space="preserve">Research/Icons/f5d3c19ee35f34a7dae4a36e5ec57472[PictoIcon_Boss]</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G52">
         <v>5</v>
       </c>
-      <c r="G52">
+      <c r="H52">
         <v>0.02</v>
       </c>
-      <c r="H52">
+      <c r="I52">
         <v>6</v>
       </c>
-      <c r="I52">
+      <c r="J52">
         <v>-1</v>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t xml:space="preserve">2-L2</t>
         </is>
       </c>
-      <c r="K52">
-        <v>0</v>
-      </c>
       <c r="L52">
         <v>0</v>
       </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N52">
+      <c r="M52">
+        <v>0</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O52">
         <v>19</v>
       </c>
     </row>
@@ -3173,38 +3433,43 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F53">
+          <t xml:space="preserve">Research/Icons/a5edbb1acb3234a5db0f0daa141eb77b[PictoIcon_Fire]</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G53">
         <v>5</v>
       </c>
-      <c r="G53">
+      <c r="H53">
         <v>0.01</v>
       </c>
-      <c r="H53">
+      <c r="I53">
         <v>6</v>
       </c>
-      <c r="I53">
-        <v>0</v>
-      </c>
-      <c r="J53" t="inlineStr">
+      <c r="J53">
+        <v>0</v>
+      </c>
+      <c r="K53" t="inlineStr">
         <is>
           <t xml:space="preserve">2-M2</t>
         </is>
       </c>
-      <c r="K53">
-        <v>0</v>
-      </c>
       <c r="L53">
         <v>0</v>
       </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N53">
+      <c r="M53">
+        <v>0</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O53">
         <v>20</v>
       </c>
     </row>
@@ -3231,38 +3496,43 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F54">
+          <t xml:space="preserve">Research/Icons/1e41e49e206bc2947b8943351eed53d3[Clock]</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G54">
         <v>5</v>
       </c>
-      <c r="G54">
+      <c r="H54">
         <v>0.03</v>
       </c>
-      <c r="H54">
+      <c r="I54">
         <v>6</v>
       </c>
-      <c r="I54">
+      <c r="J54">
         <v>1</v>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t xml:space="preserve">2-R2</t>
         </is>
       </c>
-      <c r="K54">
-        <v>0</v>
-      </c>
       <c r="L54">
         <v>0</v>
       </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N54">
+      <c r="M54">
+        <v>0</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O54">
         <v>21</v>
       </c>
     </row>
@@ -3289,38 +3559,43 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/038ccab8cd184d04cb1bfa1d79704320[Medal]</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
           <t xml:space="preserve">Circle</t>
         </is>
       </c>
-      <c r="F55">
+      <c r="G55">
         <v>1</v>
       </c>
-      <c r="G55">
+      <c r="H55">
         <v>0.05</v>
       </c>
-      <c r="H55">
+      <c r="I55">
         <v>7</v>
       </c>
-      <c r="I55">
-        <v>0</v>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K55">
-        <v>0</v>
+      <c r="J55">
+        <v>0</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="L55">
+        <v>0</v>
+      </c>
+      <c r="M55">
         <v>40</v>
       </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N55">
+      <c r="N55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O55">
         <v>23</v>
       </c>
     </row>
@@ -3347,38 +3622,43 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F56">
+          <t xml:space="preserve">Research/Icons/f9b293277bc1b4e24b12ba67c353239b[PictoIcon_Attack_Power]</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G56">
         <v>5</v>
       </c>
-      <c r="G56">
+      <c r="H56">
         <v>0.02</v>
       </c>
-      <c r="H56">
+      <c r="I56">
         <v>8</v>
       </c>
-      <c r="I56">
+      <c r="J56">
         <v>-1</v>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t xml:space="preserve">G2</t>
         </is>
       </c>
-      <c r="K56">
-        <v>0</v>
-      </c>
       <c r="L56">
         <v>0</v>
       </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N56">
+      <c r="M56">
+        <v>0</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O56">
         <v>25</v>
       </c>
     </row>
@@ -3405,38 +3685,43 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F57">
+          <t xml:space="preserve">Research/Icons/e0d9939b4e24549aebfe1441f4104b8b[PictoIcon_Critical]</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G57">
         <v>5</v>
       </c>
-      <c r="G57">
+      <c r="H57">
         <v>0.01</v>
       </c>
-      <c r="H57">
+      <c r="I57">
         <v>8</v>
       </c>
-      <c r="I57">
-        <v>0</v>
-      </c>
-      <c r="J57" t="inlineStr">
+      <c r="J57">
+        <v>0</v>
+      </c>
+      <c r="K57" t="inlineStr">
         <is>
           <t xml:space="preserve">G2</t>
         </is>
       </c>
-      <c r="K57">
-        <v>0</v>
-      </c>
       <c r="L57">
         <v>0</v>
       </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N57">
+      <c r="M57">
+        <v>0</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O57">
         <v>26</v>
       </c>
     </row>
@@ -3463,38 +3748,43 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F58">
+          <t xml:space="preserve">Research/Icons/447cb81759d8742888a02fa6be150fd0[PictoIcon_Support]</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G58">
         <v>5</v>
       </c>
-      <c r="G58">
+      <c r="H58">
         <v>0.03</v>
       </c>
-      <c r="H58">
+      <c r="I58">
         <v>8</v>
       </c>
-      <c r="I58">
+      <c r="J58">
         <v>1</v>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t xml:space="preserve">G2</t>
         </is>
       </c>
-      <c r="K58">
-        <v>0</v>
-      </c>
       <c r="L58">
         <v>0</v>
       </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N58">
+      <c r="M58">
+        <v>0</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O58">
         <v>27</v>
       </c>
     </row>
@@ -3521,38 +3811,43 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F59">
+          <t xml:space="preserve">Research/Icons/9851fb8e6f12a40d09379e3d9a144449[PictoIcon_Thunder]</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G59">
         <v>5</v>
       </c>
-      <c r="G59">
+      <c r="H59">
         <v>0.02</v>
       </c>
-      <c r="H59">
+      <c r="I59">
         <v>9</v>
       </c>
-      <c r="I59">
+      <c r="J59">
         <v>-1</v>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="K59" t="inlineStr">
         <is>
           <t xml:space="preserve">3-L1</t>
         </is>
       </c>
-      <c r="K59">
-        <v>0</v>
-      </c>
       <c r="L59">
         <v>0</v>
       </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N59">
+      <c r="M59">
+        <v>0</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O59">
         <v>28</v>
       </c>
     </row>
@@ -3579,38 +3874,43 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F60">
+          <t xml:space="preserve">Research/Icons/9df0f4d8c02014347ad2d7de427e0ced[Star Filled]</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G60">
         <v>5</v>
       </c>
-      <c r="G60">
+      <c r="H60">
         <v>0.01</v>
       </c>
-      <c r="H60">
+      <c r="I60">
         <v>9</v>
       </c>
-      <c r="I60">
-        <v>0</v>
-      </c>
-      <c r="J60" t="inlineStr">
+      <c r="J60">
+        <v>0</v>
+      </c>
+      <c r="K60" t="inlineStr">
         <is>
           <t xml:space="preserve">3-M1</t>
         </is>
       </c>
-      <c r="K60">
-        <v>0</v>
-      </c>
       <c r="L60">
         <v>0</v>
       </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N60">
+      <c r="M60">
+        <v>0</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O60">
         <v>29</v>
       </c>
     </row>
@@ -3637,38 +3937,43 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Square</t>
-        </is>
-      </c>
-      <c r="F61">
+          <t xml:space="preserve">Research/Icons/e7f5d551fd1925040bd01a8ec66c0ae0[Store Bag]</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Square</t>
+        </is>
+      </c>
+      <c r="G61">
         <v>5</v>
       </c>
-      <c r="G61">
+      <c r="H61">
         <v>30</v>
       </c>
-      <c r="H61">
+      <c r="I61">
         <v>9</v>
       </c>
-      <c r="I61">
+      <c r="J61">
         <v>1</v>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="K61" t="inlineStr">
         <is>
           <t xml:space="preserve">3-R1</t>
         </is>
       </c>
-      <c r="K61">
-        <v>0</v>
-      </c>
       <c r="L61">
         <v>0</v>
       </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N61">
+      <c r="M61">
+        <v>0</v>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O61">
         <v>30</v>
       </c>
     </row>
@@ -3695,38 +4000,43 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
+          <t xml:space="preserve">Research/Icons/65a1928224b8541439b433a52ea9c3d9[Cup]</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
           <t xml:space="preserve">Special</t>
         </is>
       </c>
-      <c r="F62">
+      <c r="G62">
         <v>3</v>
       </c>
-      <c r="G62">
+      <c r="H62">
         <v>0.1</v>
       </c>
-      <c r="H62">
+      <c r="I62">
         <v>10</v>
       </c>
-      <c r="I62">
-        <v>0</v>
-      </c>
-      <c r="J62" t="inlineStr">
+      <c r="J62">
+        <v>0</v>
+      </c>
+      <c r="K62" t="inlineStr">
         <is>
           <t xml:space="preserve">3-L2;3-M2;3-R2</t>
         </is>
       </c>
-      <c r="K62">
-        <v>0</v>
-      </c>
       <c r="L62">
         <v>0</v>
       </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="N62">
+      <c r="M62">
+        <v>0</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O62">
         <v>32</v>
       </c>
     </row>

</xml_diff>